<commit_message>
feat(perf-strategica): scoring consuntivazione (calcolo diretto) + classificazione rapporto A/B + fix fasce
saveIndicatorConsuntivo: scoring silente al salvataggio (ACTUAL -> fascia RNG_* -> % -> x peso = SCOREKPI in punti), SI_NO per tipo. Classificazione num/den: rapporto A/B (senza x100) vs percentuale A/B*100 dal Target del master; catalogo Tipologia corretto. riconcilia_catalogo_indicatori.py tipologia() Target-based + override; genera_import_da_obiettivi.py fonde bande stesso factor (ST59/C33) + override A66. POST_IMPORT_FASCE_COMPLETO.sql rigenerato (ST59); POST_IMPORT_FIX_RAPPORTI.sql passo 4 di SETUP_POST_IMPORT.
</commit_message>
<xml_diff>
--- a/script/templates/IndicatoriCatalogo_BS.xlsx
+++ b/script/templates/IndicatoriCatalogo_BS.xlsx
@@ -1504,7 +1504,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>(A-B)/B*100</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>SI_NO</t>
+          <t>(A-B)/B*100</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3886,7 +3886,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>A/B</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -5394,6 +5394,11 @@
           <t>Promuovere le attività del gruppo di supporto alla Direzione Sanitaria per la valutazione delle tecnologie sanitarie.</t>
         </is>
       </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>A/B*100</t>
+        </is>
+      </c>
       <c r="E147" t="inlineStr">
         <is>
           <t>AREA_SERV_STR</t>
@@ -5783,7 +5788,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>SI_NO</t>
+          <t>A/B*100</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -6079,7 +6084,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>SI_NO</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -6294,11 +6299,6 @@
           <t>Piano di Formazione FSE 2.0 - intervento PNRR - Missione 6 "Salute", Componente 2 sub-investimento 1.31 (b) "Adozione e utilizzo del Fascicolo Sanitario Elettronico da parte delle Regioni - Change management"</t>
         </is>
       </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>SI_NO</t>
-        </is>
-      </c>
       <c r="E172" t="inlineStr">
         <is>
           <t>AREA_SERV_STR</t>
@@ -7563,11 +7563,6 @@
           <t>Giacenze fisiche del magazzino farmaceutico e le giacenze fisiche presso tutti i reparti dell'azienda.</t>
         </is>
       </c>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t>A/B*100</t>
-        </is>
-      </c>
       <c r="E209" t="inlineStr">
         <is>
           <t>AREA_SERV_SAN</t>
@@ -8541,7 +8536,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>A/B</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
@@ -8578,7 +8573,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>A/B</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
@@ -8615,7 +8610,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>A/B</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -11334,7 +11329,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>A/B</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -13327,7 +13322,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>SI_NO</t>
         </is>
       </c>
       <c r="E377" t="inlineStr">
@@ -13682,7 +13677,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>A/B</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
@@ -13719,7 +13714,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>A/B</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
@@ -13822,7 +13817,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>SUM(A)</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
@@ -14029,7 +14024,7 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>A/B*100</t>
+          <t>A/B</t>
         </is>
       </c>
       <c r="E397" t="inlineStr">

</xml_diff>